<commit_message>
Toplu veri güncelleme (yerel, 17.09.2026 17:13)
</commit_message>
<xml_diff>
--- a/kredi mevduat/kredi_mevduat.xlsx
+++ b/kredi mevduat/kredi_mevduat.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H611"/>
+  <dimension ref="A1:H612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16336,6 +16336,32 @@
       </c>
       <c r="H611" t="n">
         <v>8.15</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B612" t="n">
+        <v>64.14</v>
+      </c>
+      <c r="C612" t="n">
+        <v>40.53</v>
+      </c>
+      <c r="D612" t="n">
+        <v>41.93</v>
+      </c>
+      <c r="E612" t="n">
+        <v>53.64</v>
+      </c>
+      <c r="F612" t="n">
+        <v>63.81</v>
+      </c>
+      <c r="G612" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="H612" t="n">
+        <v>8.050000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -16349,7 +16375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K611"/>
+  <dimension ref="A1:K612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37757,6 +37783,41 @@
       </c>
       <c r="K611" t="n">
         <v>2.8</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B612" t="n">
+        <v>43.92</v>
+      </c>
+      <c r="C612" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="D612" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="E612" t="n">
+        <v>38.86</v>
+      </c>
+      <c r="F612" t="n">
+        <v>38</v>
+      </c>
+      <c r="G612" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="H612" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I612" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="J612" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="K612" t="n">
+        <v>2.72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (01.10.2026 17:32 UTC)
</commit_message>
<xml_diff>
--- a/kredi mevduat/kredi_mevduat.xlsx
+++ b/kredi mevduat/kredi_mevduat.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H613"/>
+  <dimension ref="A1:H614"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16376,6 +16376,32 @@
       </c>
       <c r="H613" t="n">
         <v>7.93</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B614" t="n">
+        <v>62.73</v>
+      </c>
+      <c r="C614" t="n">
+        <v>47.71</v>
+      </c>
+      <c r="D614" t="n">
+        <v>41.82</v>
+      </c>
+      <c r="E614" t="n">
+        <v>52.28</v>
+      </c>
+      <c r="F614" t="n">
+        <v>62.69</v>
+      </c>
+      <c r="G614" t="n">
+        <v>6.96</v>
+      </c>
+      <c r="H614" t="n">
+        <v>8.41</v>
       </c>
     </row>
   </sheetData>
@@ -16389,7 +16415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K613"/>
+  <dimension ref="A1:K614"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37867,6 +37893,41 @@
       </c>
       <c r="K613" t="n">
         <v>2.75</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B614" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="C614" t="n">
+        <v>43.77</v>
+      </c>
+      <c r="D614" t="n">
+        <v>43.17</v>
+      </c>
+      <c r="E614" t="n">
+        <v>39.81</v>
+      </c>
+      <c r="F614" t="n">
+        <v>31.32</v>
+      </c>
+      <c r="G614" t="n">
+        <v>43.35</v>
+      </c>
+      <c r="H614" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="I614" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="J614" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="K614" t="n">
+        <v>2.73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>